<commit_message>
Update AST schedule data
</commit_message>
<xml_diff>
--- a/data/DATA_AST_LSI.xlsx
+++ b/data/DATA_AST_LSI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftarr Hendry\Documents\annual_stock_take\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FB41FC-D8A0-4C4D-B377-FCCBBDD8B815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25C89E9-D1A7-4C39-96C1-E3F5E559566C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{359B9B45-F88B-4FAF-99A8-60573E35A8DF}"/>
   </bookViews>
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="159">
   <si>
     <t>BATCH</t>
   </si>
@@ -668,6 +668,9 @@
   </si>
   <si>
     <t>kaisar rauf pasha</t>
+  </si>
+  <si>
+    <t>60023</t>
   </si>
 </sst>
 </file>
@@ -679,7 +682,7 @@
     <numFmt numFmtId="165" formatCode="#,##0;[Black]&quot;▲&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0;[Black]&quot;▲&quot;#,##0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -749,6 +752,13 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="NanumBarunGothicOTF"/>
+      <family val="1"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="6">
@@ -882,7 +892,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -983,9 +993,27 @@
     <xf numFmtId="16" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -998,22 +1026,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1421,7 +1440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E9D3950-46A3-4710-8283-CFEB8F7F9459}">
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P60"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="6.5546875" bestFit="1" customWidth="1"/>
@@ -1441,44 +1460,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="36" t="s">
+      <c r="C1" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="38" t="s">
+      <c r="D1" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="44">
+      <c r="E1" s="40">
         <v>2026</v>
       </c>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="41" t="s">
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="41" t="s">
+      <c r="I1" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="42" t="s">
+      <c r="J1" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
     </row>
     <row r="2" spans="1:16" ht="34.799999999999997">
-      <c r="A2" s="35"/>
-      <c r="B2" s="35"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="38"/>
+      <c r="A2" s="41"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="44"/>
       <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1488,8 +1507,8 @@
       <c r="G2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
       <c r="J2" s="3" t="s">
         <v>10</v>
       </c>
@@ -1531,7 +1550,7 @@
       <c r="P3" s="12"/>
     </row>
     <row r="4" spans="1:16" ht="15">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="13" t="s">
@@ -1579,7 +1598,7 @@
       </c>
     </row>
     <row r="5" spans="1:16" ht="15">
-      <c r="A5" s="40"/>
+      <c r="A5" s="35"/>
       <c r="B5" s="13" t="s">
         <v>24</v>
       </c>
@@ -1693,7 +1712,7 @@
       </c>
     </row>
     <row r="8" spans="1:16" ht="15">
-      <c r="A8" s="39">
+      <c r="A8" s="34">
         <v>2</v>
       </c>
       <c r="B8" s="13" t="s">
@@ -1743,7 +1762,7 @@
       </c>
     </row>
     <row r="9" spans="1:16" ht="15">
-      <c r="A9" s="40"/>
+      <c r="A9" s="35"/>
       <c r="B9" s="13" t="s">
         <v>24</v>
       </c>
@@ -1809,17 +1828,17 @@
       <c r="P10" s="24"/>
     </row>
     <row r="11" spans="1:16" ht="15">
-      <c r="A11" s="34">
+      <c r="A11" s="36">
         <v>2</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>48</v>
+      <c r="C11" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" s="45" t="s">
+        <v>63</v>
       </c>
       <c r="E11" s="16">
         <v>46314</v>
@@ -1837,37 +1856,37 @@
         <v>46329</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="L11" s="19" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="M11" s="19" t="s">
         <v>51</v>
       </c>
       <c r="N11" s="20">
-        <v>-370</v>
+        <v>-700.12512500000003</v>
       </c>
       <c r="O11" s="20">
-        <v>-26</v>
+        <v>-1.8748749999999745</v>
       </c>
       <c r="P11" s="21">
-        <v>-6.5656565656565666</v>
+        <v>-0.26707621082620719</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="15">
-      <c r="A12" s="34"/>
+      <c r="A12" s="36"/>
       <c r="B12" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>52</v>
+      <c r="C12" s="14" t="s">
+        <v>158</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E12" s="16">
         <v>46314</v>
@@ -1885,29 +1904,29 @@
         <v>46329</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="K12" s="19" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="L12" s="19" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="M12" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="N12" s="25">
-        <v>-673</v>
+        <v>58</v>
+      </c>
+      <c r="N12" s="20">
+        <v>-599.39536959999998</v>
       </c>
       <c r="O12" s="20">
-        <v>477</v>
+        <v>-88.604630400000019</v>
       </c>
       <c r="P12" s="21">
-        <v>243.36734693877551</v>
+        <v>-12.878580000000003</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="15">
-      <c r="A13" s="34"/>
+      <c r="A13" s="36"/>
       <c r="B13" s="13" t="s">
         <v>24</v>
       </c>
@@ -1973,7 +1992,7 @@
       <c r="P14" s="24"/>
     </row>
     <row r="15" spans="1:16" ht="15">
-      <c r="A15" s="39">
+      <c r="A15" s="34">
         <v>3</v>
       </c>
       <c r="B15" s="13" t="s">
@@ -2023,15 +2042,15 @@
       </c>
     </row>
     <row r="16" spans="1:16" ht="15">
-      <c r="A16" s="40"/>
+      <c r="A16" s="35"/>
       <c r="B16" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="13" t="s">
-        <v>62</v>
+      <c r="C16" s="14" t="s">
+        <v>47</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="E16" s="16">
         <v>46319</v>
@@ -2049,25 +2068,25 @@
         <v>46334</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="L16" s="19" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="M16" s="19" t="s">
         <v>51</v>
       </c>
       <c r="N16" s="20">
-        <v>-700.12512500000003</v>
+        <v>-370</v>
       </c>
       <c r="O16" s="20">
-        <v>-1.8748749999999745</v>
+        <v>-26</v>
       </c>
       <c r="P16" s="21">
-        <v>-0.26707621082620719</v>
+        <v>-6.5656565656565666</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="15">
@@ -2077,11 +2096,11 @@
       <c r="B17" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="27">
-        <v>6023</v>
+      <c r="C17" s="47" t="s">
+        <v>52</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E17" s="16">
         <v>46344</v>
@@ -2099,25 +2118,25 @@
         <v>46359</v>
       </c>
       <c r="J17" s="19" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="K17" s="19" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="L17" s="19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="M17" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="N17" s="20">
-        <v>-599.39536959999998</v>
+        <v>46</v>
+      </c>
+      <c r="N17" s="25">
+        <v>-673</v>
       </c>
       <c r="O17" s="20">
-        <v>-88.604630400000019</v>
+        <v>477</v>
       </c>
       <c r="P17" s="21">
-        <v>-12.878580000000003</v>
+        <v>243.36734693877551</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="15">
@@ -2139,7 +2158,7 @@
       <c r="P18" s="24"/>
     </row>
     <row r="19" spans="1:16" ht="15">
-      <c r="A19" s="34">
+      <c r="A19" s="36">
         <v>3</v>
       </c>
       <c r="B19" s="13" t="s">
@@ -2189,7 +2208,7 @@
       </c>
     </row>
     <row r="20" spans="1:16" ht="15">
-      <c r="A20" s="34"/>
+      <c r="A20" s="36"/>
       <c r="B20" s="13" t="s">
         <v>24</v>
       </c>
@@ -2237,7 +2256,7 @@
       </c>
     </row>
     <row r="21" spans="1:16" ht="15">
-      <c r="A21" s="34"/>
+      <c r="A21" s="36"/>
       <c r="B21" s="13" t="s">
         <v>24</v>
       </c>
@@ -2303,7 +2322,7 @@
       <c r="P22" s="24"/>
     </row>
     <row r="23" spans="1:16" ht="15">
-      <c r="A23" s="34">
+      <c r="A23" s="36">
         <v>4</v>
       </c>
       <c r="B23" s="13" t="s">
@@ -2353,7 +2372,7 @@
       </c>
     </row>
     <row r="24" spans="1:16" ht="15">
-      <c r="A24" s="34"/>
+      <c r="A24" s="36"/>
       <c r="B24" s="13" t="s">
         <v>24</v>
       </c>
@@ -2401,7 +2420,7 @@
       </c>
     </row>
     <row r="25" spans="1:16" ht="15">
-      <c r="A25" s="34"/>
+      <c r="A25" s="36"/>
       <c r="B25" s="13" t="s">
         <v>24</v>
       </c>
@@ -2467,7 +2486,7 @@
       <c r="P26" s="24"/>
     </row>
     <row r="27" spans="1:16" ht="15">
-      <c r="A27" s="34">
+      <c r="A27" s="36">
         <v>5</v>
       </c>
       <c r="B27" s="13" t="s">
@@ -2517,7 +2536,7 @@
       </c>
     </row>
     <row r="28" spans="1:16" ht="15">
-      <c r="A28" s="34"/>
+      <c r="A28" s="36"/>
       <c r="B28" s="13" t="s">
         <v>24</v>
       </c>
@@ -2565,7 +2584,7 @@
       </c>
     </row>
     <row r="29" spans="1:16" ht="15">
-      <c r="A29" s="34"/>
+      <c r="A29" s="36"/>
       <c r="B29" s="13" t="s">
         <v>24</v>
       </c>
@@ -2631,7 +2650,7 @@
       <c r="P30" s="24"/>
     </row>
     <row r="31" spans="1:16" ht="15">
-      <c r="A31" s="34">
+      <c r="A31" s="36">
         <v>6</v>
       </c>
       <c r="B31" s="13" t="s">
@@ -2681,7 +2700,7 @@
       </c>
     </row>
     <row r="32" spans="1:16" ht="15">
-      <c r="A32" s="34"/>
+      <c r="A32" s="36"/>
       <c r="B32" s="13" t="s">
         <v>24</v>
       </c>
@@ -2729,7 +2748,7 @@
       </c>
     </row>
     <row r="33" spans="1:16" ht="15">
-      <c r="A33" s="34"/>
+      <c r="A33" s="36"/>
       <c r="B33" s="13" t="s">
         <v>24</v>
       </c>
@@ -2795,7 +2814,7 @@
       <c r="P34" s="24"/>
     </row>
     <row r="35" spans="1:16" ht="15">
-      <c r="A35" s="34">
+      <c r="A35" s="36">
         <v>7</v>
       </c>
       <c r="B35" s="13" t="s">
@@ -2845,7 +2864,7 @@
       </c>
     </row>
     <row r="36" spans="1:16" ht="15">
-      <c r="A36" s="34"/>
+      <c r="A36" s="36"/>
       <c r="B36" s="13" t="s">
         <v>24</v>
       </c>
@@ -2893,7 +2912,7 @@
       </c>
     </row>
     <row r="37" spans="1:16" ht="15">
-      <c r="A37" s="34"/>
+      <c r="A37" s="36"/>
       <c r="B37" s="13" t="s">
         <v>24</v>
       </c>
@@ -2959,7 +2978,7 @@
       <c r="P38" s="24"/>
     </row>
     <row r="39" spans="1:16" ht="15">
-      <c r="A39" s="34">
+      <c r="A39" s="36">
         <v>8</v>
       </c>
       <c r="B39" s="13" t="s">
@@ -3009,7 +3028,7 @@
       </c>
     </row>
     <row r="40" spans="1:16" ht="15">
-      <c r="A40" s="34"/>
+      <c r="A40" s="36"/>
       <c r="B40" s="13" t="s">
         <v>24</v>
       </c>
@@ -3057,7 +3076,7 @@
       </c>
     </row>
     <row r="41" spans="1:16" ht="15">
-      <c r="A41" s="34"/>
+      <c r="A41" s="36"/>
       <c r="B41" s="13" t="s">
         <v>24</v>
       </c>
@@ -3123,7 +3142,7 @@
       <c r="P42" s="24"/>
     </row>
     <row r="43" spans="1:16" ht="15">
-      <c r="A43" s="34">
+      <c r="A43" s="36">
         <v>9</v>
       </c>
       <c r="B43" s="13" t="s">
@@ -3173,7 +3192,7 @@
       </c>
     </row>
     <row r="44" spans="1:16" ht="15">
-      <c r="A44" s="34"/>
+      <c r="A44" s="36"/>
       <c r="B44" s="13" t="s">
         <v>24</v>
       </c>
@@ -3221,7 +3240,7 @@
       </c>
     </row>
     <row r="45" spans="1:16" ht="15">
-      <c r="A45" s="34"/>
+      <c r="A45" s="36"/>
       <c r="B45" s="13" t="s">
         <v>24</v>
       </c>
@@ -3287,7 +3306,7 @@
       <c r="P46" s="24"/>
     </row>
     <row r="47" spans="1:16" ht="15">
-      <c r="A47" s="34">
+      <c r="A47" s="36">
         <v>10</v>
       </c>
       <c r="B47" s="13" t="s">
@@ -3337,7 +3356,7 @@
       </c>
     </row>
     <row r="48" spans="1:16" ht="15">
-      <c r="A48" s="34"/>
+      <c r="A48" s="36"/>
       <c r="B48" s="13" t="s">
         <v>24</v>
       </c>
@@ -3385,7 +3404,7 @@
       </c>
     </row>
     <row r="49" spans="1:16" ht="15">
-      <c r="A49" s="34"/>
+      <c r="A49" s="36"/>
       <c r="B49" s="13" t="s">
         <v>24</v>
       </c>
@@ -3451,7 +3470,7 @@
       <c r="P50" s="24"/>
     </row>
     <row r="51" spans="1:16" ht="15">
-      <c r="A51" s="34">
+      <c r="A51" s="36">
         <v>11</v>
       </c>
       <c r="B51" s="13" t="s">
@@ -3501,7 +3520,7 @@
       </c>
     </row>
     <row r="52" spans="1:16" ht="15">
-      <c r="A52" s="34"/>
+      <c r="A52" s="36"/>
       <c r="B52" s="13" t="s">
         <v>24</v>
       </c>
@@ -3549,7 +3568,7 @@
       </c>
     </row>
     <row r="53" spans="1:16" ht="15">
-      <c r="A53" s="34"/>
+      <c r="A53" s="36"/>
       <c r="B53" s="13" t="s">
         <v>24</v>
       </c>
@@ -3614,8 +3633,87 @@
       <c r="O54" s="23"/>
       <c r="P54" s="24"/>
     </row>
+    <row r="56" spans="1:16" ht="15">
+      <c r="B56" s="13"/>
+      <c r="C56" s="13"/>
+      <c r="D56" s="46"/>
+      <c r="E56" s="16"/>
+      <c r="F56" s="17"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="17"/>
+      <c r="I56" s="17"/>
+      <c r="J56" s="19"/>
+      <c r="K56" s="19"/>
+      <c r="L56" s="19"/>
+      <c r="M56" s="19"/>
+      <c r="N56" s="20"/>
+      <c r="O56" s="20"/>
+      <c r="P56" s="21"/>
+    </row>
+    <row r="57" spans="1:16" ht="15">
+      <c r="B57" s="13"/>
+      <c r="C57" s="13"/>
+      <c r="E57" s="16"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="17"/>
+      <c r="I57" s="17"/>
+      <c r="J57" s="19"/>
+      <c r="K57" s="19"/>
+      <c r="L57" s="19"/>
+      <c r="M57" s="19"/>
+      <c r="N57" s="25"/>
+      <c r="O57" s="20"/>
+      <c r="P57" s="21"/>
+    </row>
+    <row r="59" spans="1:16" ht="15">
+      <c r="B59" s="13"/>
+      <c r="C59" s="13"/>
+      <c r="D59" s="46"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="17"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="17"/>
+      <c r="I59" s="17"/>
+      <c r="J59" s="19"/>
+      <c r="K59" s="19"/>
+      <c r="L59" s="19"/>
+      <c r="M59" s="19"/>
+      <c r="N59" s="20"/>
+      <c r="O59" s="20"/>
+      <c r="P59" s="21"/>
+    </row>
+    <row r="60" spans="1:16" ht="15">
+      <c r="B60" s="13"/>
+      <c r="C60" s="27"/>
+      <c r="D60" s="46"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="17"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="17"/>
+      <c r="I60" s="17"/>
+      <c r="J60" s="19"/>
+      <c r="K60" s="19"/>
+      <c r="L60" s="19"/>
+      <c r="M60" s="19"/>
+      <c r="N60" s="20"/>
+      <c r="O60" s="20"/>
+      <c r="P60" s="21"/>
+    </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:H2"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A39:A41"/>
     <mergeCell ref="A43:A45"/>
@@ -3626,18 +3724,6 @@
     <mergeCell ref="A27:A29"/>
     <mergeCell ref="A31:A33"/>
     <mergeCell ref="A35:A37"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="A8:A9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -3645,7 +3731,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="10" operator="containsText" id="{1A0E45CE-F7AE-4D99-91A7-4F37B9FD5A27}">
+          <x14:cfRule type="containsText" priority="17" operator="containsText" id="{1A0E45CE-F7AE-4D99-91A7-4F37B9FD5A27}">
             <xm:f>NOT(ISERROR(SEARCH($D$2,A3)))</xm:f>
             <xm:f>$D$2</xm:f>
             <x14:dxf>
@@ -3656,11 +3742,11 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>A18:P54 A3:P7 B9:F9 A10:P10 A11:F13 H11:P12 H13:I13 A8:F8 H8:P9 B16:P16 A14:P14 A15:I15 K15:P15 A17:I17</xm:sqref>
+          <xm:sqref>A3:P7 A8:F8 B9:F9 B16:I16 B57:C57 E57:P57 B56:P56</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="9" operator="containsText" id="{7E5347F1-C59B-49F2-A486-348876D00DDC}">
-            <xm:f>NOT(ISERROR(SEARCH($D$2,J13)))</xm:f>
+          <x14:cfRule type="containsText" priority="9" operator="containsText" id="{949D15F9-932E-41EA-B4DC-A7B149A7FBCA}">
+            <xm:f>NOT(ISERROR(SEARCH($D$2,A10)))</xm:f>
             <xm:f>$D$2</xm:f>
             <x14:dxf>
               <fill>
@@ -3670,11 +3756,11 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>J13:P13</xm:sqref>
+          <xm:sqref>A10:P10 A13:P15 A11:I12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="8" operator="containsText" id="{4F44122A-18C2-4992-B10B-86C31D8F76CE}">
-            <xm:f>NOT(ISERROR(SEARCH($D$2,G11)))</xm:f>
+          <x14:cfRule type="containsText" priority="8" operator="containsText" id="{4FB9DF6C-0043-478D-9ED6-EFE99F22D9A1}">
+            <xm:f>NOT(ISERROR(SEARCH($D$2,A17)))</xm:f>
             <xm:f>$D$2</xm:f>
             <x14:dxf>
               <fill>
@@ -3684,52 +3770,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G11</xm:sqref>
+          <xm:sqref>A18:P54 A17:I17</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="7" operator="containsText" id="{F210AB3F-B6EF-4F37-9D77-52D955C54013}">
-            <xm:f>NOT(ISERROR(SEARCH($D$2,G12)))</xm:f>
-            <xm:f>$D$2</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFFF00"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G12</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="6" operator="containsText" id="{975E79EC-1C64-4465-9393-7FF32A205188}">
-            <xm:f>NOT(ISERROR(SEARCH($D$2,G13)))</xm:f>
-            <xm:f>$D$2</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFFF00"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G13</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{06AB4D8A-DBC1-4013-AFD7-E3C16F8D4AD8}">
-            <xm:f>NOT(ISERROR(SEARCH($D$2,G9)))</xm:f>
-            <xm:f>$D$2</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFFF00"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G9</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{6EA13ADB-3188-4884-A67E-794CFD474769}">
+          <x14:cfRule type="containsText" priority="11" operator="containsText" id="{6EA13ADB-3188-4884-A67E-794CFD474769}">
             <xm:f>NOT(ISERROR(SEARCH($D$2,G8)))</xm:f>
             <xm:f>$D$2</xm:f>
             <x14:dxf>
@@ -3740,11 +3784,11 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>G8</xm:sqref>
+          <xm:sqref>G8:P9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{949D15F9-932E-41EA-B4DC-A7B149A7FBCA}">
-            <xm:f>NOT(ISERROR(SEARCH($D$2,J15)))</xm:f>
+          <x14:cfRule type="containsText" priority="6" operator="containsText" id="{D3EBB924-75D8-469B-8C3A-A8331CEF83C2}">
+            <xm:f>NOT(ISERROR(SEARCH($D$2,B59)))</xm:f>
             <xm:f>$D$2</xm:f>
             <x14:dxf>
               <fill>
@@ -3754,10 +3798,52 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>J15</xm:sqref>
+          <xm:sqref>B59:P59</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{4FB9DF6C-0043-478D-9ED6-EFE99F22D9A1}">
+          <x14:cfRule type="containsText" priority="5" operator="containsText" id="{67CF2A4D-9843-4437-BE02-F20BF883A04D}">
+            <xm:f>NOT(ISERROR(SEARCH($D$2,B60)))</xm:f>
+            <xm:f>$D$2</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFFF00"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>B60:P60</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{9E4CEA65-8C41-4231-A737-92A79332793E}">
+            <xm:f>NOT(ISERROR(SEARCH($D$2,J11)))</xm:f>
+            <xm:f>$D$2</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFFF00"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>J11:P11</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{97C4B32D-80E9-4D03-AA73-7C7279B2EA70}">
+            <xm:f>NOT(ISERROR(SEARCH($D$2,J16)))</xm:f>
+            <xm:f>$D$2</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFFF00"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>J16:P16</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{82203E34-7862-46AC-B05E-E4A35CE202DD}">
             <xm:f>NOT(ISERROR(SEARCH($D$2,J17)))</xm:f>
             <xm:f>$D$2</xm:f>
             <x14:dxf>
@@ -3770,6 +3856,20 @@
           </x14:cfRule>
           <xm:sqref>J17:P17</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{C9F8E0B8-5BBA-4903-91BF-7F7022CD45AB}">
+            <xm:f>NOT(ISERROR(SEARCH($D$2,J12)))</xm:f>
+            <xm:f>$D$2</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFFF00"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>J12:P12</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>

</xml_diff>